<commit_message>
Changed blob detection test results to correctly display blobs detected and modules localized
</commit_message>
<xml_diff>
--- a/test/BlobDetection_test.xlsx
+++ b/test/BlobDetection_test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rasmuslykke/Desktop/P2_Battery_Disassembly/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ABCA56E-917A-A44D-BFEB-3E82C90E3AC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F85A10DE-44E9-4D43-8A56-AF7E57101068}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{6F186ABD-F6A9-D349-A0FF-ED0D3DE47F94}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16980" xr2:uid="{6F186ABD-F6A9-D349-A0FF-ED0D3DE47F94}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -39,21 +39,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>Blob Detection</t>
-  </si>
-  <si>
-    <t>Succes</t>
-  </si>
-  <si>
-    <t>Fail</t>
   </si>
   <si>
     <t>Blob Tuning</t>
   </si>
   <si>
-    <t>✓</t>
+    <t>Blobs detected</t>
+  </si>
+  <si>
+    <t>Modules Localized</t>
   </si>
 </sst>
 </file>
@@ -524,7 +521,8 @@
   <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
@@ -534,59 +532,69 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>3</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="4">
         <v>1</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="6"/>
+      <c r="B3" s="5">
+        <v>8</v>
+      </c>
+      <c r="C3" s="6">
+        <v>8</v>
+      </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="4">
         <v>2</v>
       </c>
-      <c r="B4" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="6"/>
+      <c r="B4" s="5">
+        <v>8</v>
+      </c>
+      <c r="C4" s="6">
+        <v>8</v>
+      </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="4">
         <v>3</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="6"/>
+      <c r="B5" s="5">
+        <v>8</v>
+      </c>
+      <c r="C5" s="6">
+        <v>8</v>
+      </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="4">
         <v>4</v>
       </c>
-      <c r="B6" s="5"/>
-      <c r="C6" s="6" t="s">
-        <v>4</v>
+      <c r="B6" s="5">
+        <v>6</v>
+      </c>
+      <c r="C6" s="6">
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="7">
         <v>5</v>
       </c>
-      <c r="B7" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" s="9"/>
+      <c r="B7" s="8">
+        <v>8</v>
+      </c>
+      <c r="C7" s="9">
+        <v>8</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>